<commit_message>
Safety: ASMIS # in lists, search, drawer, exports; Save with data (offline single file with embedded records); real-data commit guards
</commit_message>
<xml_diff>
--- a/dashboards/safety/data/asmis_sample.xlsx
+++ b/dashboards/safety/data/asmis_sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ASMIS Export" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Strength" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASMIS Export" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strength" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29375,11 +29375,6 @@
           <t>26-2457</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>2026758990</t>
-        </is>
-      </c>
       <c r="D147" t="inlineStr">
         <is>
           <t>Brigade Safety Officer</t>
@@ -29775,11 +29770,6 @@
           <t>27-4026</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>2026910827</t>
-        </is>
-      </c>
       <c r="D149" t="inlineStr">
         <is>
           <t>State Safety Specialist</t>
@@ -30165,11 +30155,6 @@
       <c r="B151" t="inlineStr">
         <is>
           <t>27-3963</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>2026347012</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">

</xml_diff>